<commit_message>
E2E artefacts from the post-deletion sweep
Screenshots from the full 40-script run against the build with both importers
deleted. Squashed from the five churn commits the run produced turn by turn.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/docs/client-report/reports/INVENTORY_REPORT_ALL_TIME.xlsx
+++ b/docs/client-report/reports/INVENTORY_REPORT_ALL_TIME.xlsx
@@ -680,7 +680,7 @@
         <v>15</v>
       </c>
       <c r="L2">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -718,7 +718,7 @@
         <v>15</v>
       </c>
       <c r="L3">
-        <v>14</v>
+        <v>17</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -756,7 +756,7 @@
         <v>15</v>
       </c>
       <c r="L4">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="5" spans="1:12" x14ac:dyDescent="0.25">
@@ -794,7 +794,7 @@
         <v>15</v>
       </c>
       <c r="L5">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="6" spans="1:12" x14ac:dyDescent="0.25">
@@ -832,7 +832,7 @@
         <v>15</v>
       </c>
       <c r="L6">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="7" spans="1:12" x14ac:dyDescent="0.25">
@@ -870,7 +870,7 @@
         <v>15</v>
       </c>
       <c r="L7">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8" spans="1:12" x14ac:dyDescent="0.25">
@@ -908,7 +908,7 @@
         <v>15</v>
       </c>
       <c r="L8">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="9" spans="1:12" x14ac:dyDescent="0.25">
@@ -946,7 +946,7 @@
         <v>15</v>
       </c>
       <c r="L9">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="10" spans="1:12" x14ac:dyDescent="0.25">
@@ -984,7 +984,7 @@
         <v>15</v>
       </c>
       <c r="L10">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>
@@ -1079,7 +1079,7 @@
         <v>15</v>
       </c>
       <c r="L2">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -1117,7 +1117,7 @@
         <v>15</v>
       </c>
       <c r="L3">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
     <row r="4" spans="1:12" x14ac:dyDescent="0.25">
@@ -1155,7 +1155,7 @@
         <v>15</v>
       </c>
       <c r="L4">
-        <v>38</v>
+        <v>41</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Anchor the export menu, and adopt held models on the Temu path too
e2eExportAllTimeReports  0 -> 9/9. Its download() matched the menu name
unanchored, so "Inventory Report" also matched the header's "Import
Inventory Report" and opened the importer; and it clicked the trigger once,
which ReportRangeMenu's local open state does not survive a store re-render.
Anchored and retried, same shape as the other report helpers.

e2eTemuMarketplace  0 -> 17/21. It spells the button /Load [\d,]+ rows?/
with an optional s, so the earlier adoptHeldModels pass did not match it.
Remaining four failures are its own and diagnosed next.

Suite total 708/731 -> 753/780.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T4LurPsVU5WNa1i8str9pz
</commit_message>
<xml_diff>
--- a/docs/client-report/reports/INVENTORY_REPORT_ALL_TIME.xlsx
+++ b/docs/client-report/reports/INVENTORY_REPORT_ALL_TIME.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="60">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="175" uniqueCount="63">
   <si>
     <t>Stock In Date</t>
   </si>
@@ -51,6 +51,9 @@
     <t>Age (days)</t>
   </si>
   <si>
+    <t>Return Date</t>
+  </si>
+  <si>
     <t>2026-07-25</t>
   </si>
   <si>
@@ -138,7 +141,13 @@
     <t>350000000000401</t>
   </si>
   <si>
+    <t>2026-07-21</t>
+  </si>
+  <si>
     <t>350000000000403</t>
+  </si>
+  <si>
+    <t>2026-07-23</t>
   </si>
   <si>
     <t>IPHONE 13 PRO</t>
@@ -597,17 +606,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L10"/>
+  <dimension ref="A1:M10"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="12" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -644,351 +653,381 @@
       <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="C2" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2">
         <v>320</v>
       </c>
       <c r="J2" t="s">
+        <v>20</v>
+      </c>
+      <c r="K2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L2">
+        <v>46</v>
+      </c>
+      <c r="M2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>13</v>
+      </c>
+      <c r="B3" t="s">
+        <v>14</v>
+      </c>
+      <c r="C3" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" t="s">
+        <v>16</v>
+      </c>
+      <c r="E3" t="s">
+        <v>17</v>
+      </c>
+      <c r="F3" t="s">
+        <v>16</v>
+      </c>
+      <c r="G3" t="s">
+        <v>22</v>
+      </c>
+      <c r="H3" t="s">
         <v>19</v>
-      </c>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>12</v>
-      </c>
-      <c r="B3" t="s">
-        <v>13</v>
-      </c>
-      <c r="C3" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" t="s">
-        <v>16</v>
-      </c>
-      <c r="F3" t="s">
-        <v>15</v>
-      </c>
-      <c r="G3" t="s">
-        <v>21</v>
-      </c>
-      <c r="H3" t="s">
-        <v>18</v>
       </c>
       <c r="I3">
         <v>318</v>
       </c>
       <c r="J3" t="s">
+        <v>20</v>
+      </c>
+      <c r="K3" t="s">
+        <v>16</v>
+      </c>
+      <c r="L3">
+        <v>46</v>
+      </c>
+      <c r="M3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>23</v>
+      </c>
+      <c r="B4" t="s">
+        <v>24</v>
+      </c>
+      <c r="C4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D4" t="s">
+        <v>16</v>
+      </c>
+      <c r="E4" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" t="s">
+        <v>16</v>
+      </c>
+      <c r="G4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H4" t="s">
         <v>19</v>
-      </c>
-      <c r="K3" t="s">
-        <v>15</v>
-      </c>
-      <c r="L3">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>22</v>
-      </c>
-      <c r="B4" t="s">
-        <v>23</v>
-      </c>
-      <c r="C4" t="s">
-        <v>24</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" t="s">
-        <v>15</v>
-      </c>
-      <c r="G4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H4" t="s">
-        <v>18</v>
       </c>
       <c r="I4">
         <v>205</v>
       </c>
       <c r="J4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L4">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+      <c r="M4" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F5" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G5" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="H5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I5">
         <v>240</v>
       </c>
       <c r="J5" t="s">
+        <v>20</v>
+      </c>
+      <c r="K5" t="s">
+        <v>16</v>
+      </c>
+      <c r="L5">
+        <v>70</v>
+      </c>
+      <c r="M5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>23</v>
+      </c>
+      <c r="B6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C6" t="s">
+        <v>33</v>
+      </c>
+      <c r="D6" t="s">
+        <v>16</v>
+      </c>
+      <c r="E6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F6" t="s">
+        <v>16</v>
+      </c>
+      <c r="G6" t="s">
+        <v>35</v>
+      </c>
+      <c r="H6" t="s">
         <v>19</v>
-      </c>
-      <c r="K5" t="s">
-        <v>15</v>
-      </c>
-      <c r="L5">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>22</v>
-      </c>
-      <c r="B6" t="s">
-        <v>31</v>
-      </c>
-      <c r="C6" t="s">
-        <v>32</v>
-      </c>
-      <c r="D6" t="s">
-        <v>15</v>
-      </c>
-      <c r="E6" t="s">
-        <v>33</v>
-      </c>
-      <c r="F6" t="s">
-        <v>15</v>
-      </c>
-      <c r="G6" t="s">
-        <v>34</v>
-      </c>
-      <c r="H6" t="s">
-        <v>18</v>
       </c>
       <c r="I6">
         <v>480</v>
       </c>
       <c r="J6" t="s">
+        <v>20</v>
+      </c>
+      <c r="K6" t="s">
+        <v>16</v>
+      </c>
+      <c r="L6">
+        <v>70</v>
+      </c>
+      <c r="M6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="7" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>23</v>
+      </c>
+      <c r="B7" t="s">
+        <v>36</v>
+      </c>
+      <c r="C7" t="s">
+        <v>37</v>
+      </c>
+      <c r="D7" t="s">
+        <v>38</v>
+      </c>
+      <c r="E7" t="s">
+        <v>17</v>
+      </c>
+      <c r="F7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G7" t="s">
+        <v>39</v>
+      </c>
+      <c r="H7" t="s">
         <v>19</v>
-      </c>
-      <c r="K6" t="s">
-        <v>15</v>
-      </c>
-      <c r="L6">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>22</v>
-      </c>
-      <c r="B7" t="s">
-        <v>35</v>
-      </c>
-      <c r="C7" t="s">
-        <v>36</v>
-      </c>
-      <c r="D7" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" t="s">
-        <v>16</v>
-      </c>
-      <c r="F7" t="s">
-        <v>15</v>
-      </c>
-      <c r="G7" t="s">
-        <v>38</v>
-      </c>
-      <c r="H7" t="s">
-        <v>18</v>
       </c>
       <c r="I7">
         <v>620</v>
       </c>
       <c r="J7" t="s">
+        <v>20</v>
+      </c>
+      <c r="K7" t="s">
+        <v>16</v>
+      </c>
+      <c r="L7">
+        <v>70</v>
+      </c>
+      <c r="M7" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>36</v>
+      </c>
+      <c r="C8" t="s">
+        <v>40</v>
+      </c>
+      <c r="D8" t="s">
+        <v>38</v>
+      </c>
+      <c r="E8" t="s">
+        <v>17</v>
+      </c>
+      <c r="F8" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" t="s">
+        <v>27</v>
+      </c>
+      <c r="H8" t="s">
         <v>19</v>
-      </c>
-      <c r="K7" t="s">
-        <v>15</v>
-      </c>
-      <c r="L7">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>22</v>
-      </c>
-      <c r="B8" t="s">
-        <v>35</v>
-      </c>
-      <c r="C8" t="s">
-        <v>39</v>
-      </c>
-      <c r="D8" t="s">
-        <v>37</v>
-      </c>
-      <c r="E8" t="s">
-        <v>16</v>
-      </c>
-      <c r="F8" t="s">
-        <v>15</v>
-      </c>
-      <c r="G8" t="s">
-        <v>26</v>
-      </c>
-      <c r="H8" t="s">
-        <v>18</v>
       </c>
       <c r="I8">
         <v>615</v>
       </c>
       <c r="J8" t="s">
+        <v>20</v>
+      </c>
+      <c r="K8" t="s">
+        <v>16</v>
+      </c>
+      <c r="L8">
+        <v>70</v>
+      </c>
+      <c r="M8" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="9" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>24</v>
+      </c>
+      <c r="C9" t="s">
+        <v>41</v>
+      </c>
+      <c r="D9" t="s">
+        <v>16</v>
+      </c>
+      <c r="E9" t="s">
+        <v>26</v>
+      </c>
+      <c r="F9" t="s">
+        <v>16</v>
+      </c>
+      <c r="G9" t="s">
+        <v>39</v>
+      </c>
+      <c r="H9" t="s">
         <v>19</v>
-      </c>
-      <c r="K8" t="s">
-        <v>15</v>
-      </c>
-      <c r="L8">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>22</v>
-      </c>
-      <c r="B9" t="s">
-        <v>23</v>
-      </c>
-      <c r="C9" t="s">
-        <v>40</v>
-      </c>
-      <c r="D9" t="s">
-        <v>15</v>
-      </c>
-      <c r="E9" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" t="s">
-        <v>15</v>
-      </c>
-      <c r="G9" t="s">
-        <v>38</v>
-      </c>
-      <c r="H9" t="s">
-        <v>18</v>
       </c>
       <c r="I9">
         <v>200</v>
       </c>
       <c r="J9" t="s">
+        <v>20</v>
+      </c>
+      <c r="K9" t="s">
+        <v>16</v>
+      </c>
+      <c r="L9">
+        <v>70</v>
+      </c>
+      <c r="M9" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="10" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>23</v>
+      </c>
+      <c r="B10" t="s">
+        <v>32</v>
+      </c>
+      <c r="C10" t="s">
+        <v>43</v>
+      </c>
+      <c r="D10" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" t="s">
+        <v>16</v>
+      </c>
+      <c r="G10" t="s">
+        <v>39</v>
+      </c>
+      <c r="H10" t="s">
         <v>19</v>
-      </c>
-      <c r="K9" t="s">
-        <v>15</v>
-      </c>
-      <c r="L9">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>22</v>
-      </c>
-      <c r="B10" t="s">
-        <v>31</v>
-      </c>
-      <c r="C10" t="s">
-        <v>41</v>
-      </c>
-      <c r="D10" t="s">
-        <v>15</v>
-      </c>
-      <c r="E10" t="s">
-        <v>33</v>
-      </c>
-      <c r="F10" t="s">
-        <v>15</v>
-      </c>
-      <c r="G10" t="s">
-        <v>38</v>
-      </c>
-      <c r="H10" t="s">
-        <v>18</v>
       </c>
       <c r="I10">
         <v>200</v>
       </c>
       <c r="J10" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="K10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L10">
+        <v>70</v>
+      </c>
+      <c r="M10" t="s">
         <v>44</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -996,17 +1035,17 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:M4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="10" width="14" customWidth="1"/>
     <col min="11" max="11" width="30" customWidth="1"/>
-    <col min="12" max="12" width="14" customWidth="1"/>
+    <col min="12" max="13" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1043,123 +1082,135 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.25">
+      <c r="M1" s="2" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="2" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B2" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="C2" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="D2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G2" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="H2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I2">
         <v>520</v>
       </c>
       <c r="J2" t="s">
+        <v>48</v>
+      </c>
+      <c r="K2" t="s">
+        <v>16</v>
+      </c>
+      <c r="L2">
+        <v>70</v>
+      </c>
+      <c r="M2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>23</v>
+      </c>
+      <c r="B3" t="s">
         <v>45</v>
       </c>
-      <c r="K2" t="s">
-        <v>15</v>
-      </c>
-      <c r="L2">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B3" t="s">
-        <v>42</v>
-      </c>
       <c r="C3" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="D3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G3" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="H3" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="I3">
         <v>525</v>
       </c>
       <c r="J3" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="K3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L3">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.25">
+        <v>70</v>
+      </c>
+      <c r="M3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="4" spans="1:13" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B4" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="C4" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="D4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="E4" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="F4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G4" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="H4" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="I4">
         <v>430</v>
       </c>
       <c r="J4" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="K4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="L4">
-        <v>44</v>
+        <v>70</v>
+      </c>
+      <c r="M4" t="s">
+        <v>16</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L1"/>
+  <autoFilter ref="A1:M1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>
@@ -1178,19 +1229,19 @@
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C1" s="3" t="s">
         <v>7</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="F1" s="3" t="s">
         <v>8</v>
@@ -1201,16 +1252,16 @@
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>55</v>
+        <v>58</v>
       </c>
       <c r="B2" t="s">
-        <v>56</v>
+        <v>59</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D2" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E2">
         <v>46</v>
@@ -1219,21 +1270,21 @@
         <v>3.2</v>
       </c>
       <c r="G2" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>58</v>
+        <v>61</v>
       </c>
       <c r="B3" t="s">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="D3" t="s">
-        <v>57</v>
+        <v>60</v>
       </c>
       <c r="E3">
         <v>22</v>
@@ -1242,7 +1293,7 @@
         <v>1.1</v>
       </c>
       <c r="G3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
   </sheetData>

</xml_diff>